<commit_message>
Build Q2438 Kubernetes Windows task
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Rf1218f093fb844ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Rf4f9cbd3a9044492"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -290,7 +290,7 @@
         <x:v>任务ID</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
-        <x:v>kubernetes_observability_rbac_handover</x:v>
+        <x:v>kubernetes_tenant_observability_release</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -338,7 +338,7 @@
         <x:v>目标输出文件</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>output/bundle清单、output/rendered渲染结果、output/results静态评审、output/tools构建入口及output/HANDOVER.md</x:v>
+        <x:v>output/bundle清单、output/rendered渲染结果、output/results静态记录、output/tools构建入口及output/RELEASE-NOTES.md</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -346,7 +346,7 @@
         <x:v>核心操作链</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>现行问题核对→只读角色拆分→绑定范围调整→Kustomize构建→静态权限评审→现场交接</x:v>
+        <x:v>现行问题核对→只读角色拆分→绑定范围变更→Kustomize构建→静态权限核对→现场发布</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">

</xml_diff>